<commit_message>
chore(pricing): regenerated Karoo example config workbook
Left over from the pricing v2 session's example rebuild. Kept on Duncan's
instruction, 4 Sep 2026.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/pricing/Karoo_Pricing_Config.xlsx
+++ b/examples/pricing/Karoo_Pricing_Config.xlsx
@@ -1,283 +1,303 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duncan/Dev/Turas/examples/pricing/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0AC23C-8252-8D44-B167-F1725ECAE8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="20360" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="VanWestendorp" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="GaborGranger" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Validation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Settings" sheetId="1" r:id="rId1"/>
+    <sheet name="VanWestendorp" sheetId="2" r:id="rId2"/>
+    <sheet name="GaborGranger" sheetId="3" r:id="rId3"/>
+    <sheet name="Validation" sheetId="4" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
-  <si>
-    <t xml:space="preserve">Setting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project_Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karoo Coffee 250 g bag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analysis_Method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">both</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data_File</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karoo_Pricing_Data.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output_File</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output/Karoo_Pricing_Results.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_Variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RespID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight_Variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Currency_Symbol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unit_Cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DK_Codes</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Generate_HTML_Report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generate_Simulator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generate_Stats_Pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generate_Tabs_Export</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabs_Question_Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GGACC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VW_Monotonicity_Behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GG_Monotonicity_Behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">smooth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segment_Column</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min_Segment_N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Include_Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N_Tiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tier_Names</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value;Standard;Premium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min_Gap_Pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max_Gap_Pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Round_To</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyst_Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Turas example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Research_House</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Research LampPost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Col_Too_Cheap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VW_TooCheap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Col_Cheap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VW_Cheap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Col_Expensive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VW_Expensive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Col_Too_Expensive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VW_TooExpensive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculate_Confidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidence_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.95</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bootstrap_Iterations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data_Format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price_Sequence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60;80;100;120;140</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Response_Columns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GG_R60;GG_R80;GG_R100;GG_R120;GG_R140</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Response_Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">binary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoothing_Method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isotonic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculate_Elasticity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revenue_Optimization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidence_Intervals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min_Completeness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min_Sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price_Min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price_Max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">500</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Project_Name</t>
+  </si>
+  <si>
+    <t>Karoo Coffee 250 g bag</t>
+  </si>
+  <si>
+    <t>Analysis_Method</t>
+  </si>
+  <si>
+    <t>both</t>
+  </si>
+  <si>
+    <t>Data_File</t>
+  </si>
+  <si>
+    <t>Karoo_Pricing_Data.xlsx</t>
+  </si>
+  <si>
+    <t>Output_File</t>
+  </si>
+  <si>
+    <t>Output/Karoo_Pricing_Results.xlsx</t>
+  </si>
+  <si>
+    <t>ID_Variable</t>
+  </si>
+  <si>
+    <t>RespID</t>
+  </si>
+  <si>
+    <t>Weight_Variable</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Currency_Symbol</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Unit_Cost</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>DK_Codes</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Generate_HTML_Report</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>Generate_Simulator</t>
+  </si>
+  <si>
+    <t>Generate_Stats_Pack</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Generate_Tabs_Export</t>
+  </si>
+  <si>
+    <t>Tabs_Question_Code</t>
+  </si>
+  <si>
+    <t>GGACC</t>
+  </si>
+  <si>
+    <t>VW_Monotonicity_Behavior</t>
+  </si>
+  <si>
+    <t>drop</t>
+  </si>
+  <si>
+    <t>GG_Monotonicity_Behavior</t>
+  </si>
+  <si>
+    <t>smooth</t>
+  </si>
+  <si>
+    <t>Segment_Column</t>
+  </si>
+  <si>
+    <t>Segment</t>
+  </si>
+  <si>
+    <t>Min_Segment_N</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Include_Total</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>N_Tiers</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Tier_Names</t>
+  </si>
+  <si>
+    <t>Value;Standard;Premium</t>
+  </si>
+  <si>
+    <t>Min_Gap_Pct</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Max_Gap_Pct</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Round_To</t>
+  </si>
+  <si>
+    <t>0.99</t>
+  </si>
+  <si>
+    <t>Analyst_Name</t>
+  </si>
+  <si>
+    <t>Turas example</t>
+  </si>
+  <si>
+    <t>Research_House</t>
+  </si>
+  <si>
+    <t>The Research LampPost</t>
+  </si>
+  <si>
+    <t>Col_Too_Cheap</t>
+  </si>
+  <si>
+    <t>VW_TooCheap</t>
+  </si>
+  <si>
+    <t>Col_Cheap</t>
+  </si>
+  <si>
+    <t>VW_Cheap</t>
+  </si>
+  <si>
+    <t>Col_Expensive</t>
+  </si>
+  <si>
+    <t>VW_Expensive</t>
+  </si>
+  <si>
+    <t>Col_Too_Expensive</t>
+  </si>
+  <si>
+    <t>VW_TooExpensive</t>
+  </si>
+  <si>
+    <t>Calculate_Confidence</t>
+  </si>
+  <si>
+    <t>Confidence_Level</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>Bootstrap_Iterations</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>Data_Format</t>
+  </si>
+  <si>
+    <t>wide</t>
+  </si>
+  <si>
+    <t>Price_Sequence</t>
+  </si>
+  <si>
+    <t>60;80;100;120;140</t>
+  </si>
+  <si>
+    <t>Response_Columns</t>
+  </si>
+  <si>
+    <t>GG_R60;GG_R80;GG_R100;GG_R120;GG_R140</t>
+  </si>
+  <si>
+    <t>Response_Type</t>
+  </si>
+  <si>
+    <t>binary</t>
+  </si>
+  <si>
+    <t>Smoothing_Method</t>
+  </si>
+  <si>
+    <t>isotonic</t>
+  </si>
+  <si>
+    <t>Calculate_Elasticity</t>
+  </si>
+  <si>
+    <t>Revenue_Optimization</t>
+  </si>
+  <si>
+    <t>Confidence_Intervals</t>
+  </si>
+  <si>
+    <t>Min_Completeness</t>
+  </si>
+  <si>
+    <t>0.80</t>
+  </si>
+  <si>
+    <t>Min_Sample</t>
+  </si>
+  <si>
+    <t>Price_Min</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Price_Max</t>
+  </si>
+  <si>
+    <t>500</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -313,6 +333,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -594,15 +623,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="48.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="2" width="48.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -610,7 +639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -618,7 +647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -626,7 +655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -634,7 +663,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -642,7 +671,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -650,7 +679,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -658,7 +687,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -666,7 +695,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -674,7 +703,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -682,23 +711,23 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12">
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13">
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -706,7 +735,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -714,7 +743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -722,7 +751,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -730,7 +759,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -738,7 +767,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -746,7 +775,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -754,7 +783,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -762,7 +791,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -770,7 +799,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -778,7 +807,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -786,7 +815,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -794,7 +823,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -802,7 +831,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -810,7 +839,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -820,20 +849,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="48.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="2" width="48.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -841,7 +870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -849,7 +878,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -857,7 +886,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -865,7 +894,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>58</v>
       </c>
@@ -873,7 +902,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -881,7 +910,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -889,7 +918,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>63</v>
       </c>
@@ -899,20 +928,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="48.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="2" width="48.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -920,7 +949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -928,7 +957,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>67</v>
       </c>
@@ -936,7 +965,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -944,7 +973,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -952,7 +981,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -960,7 +989,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -968,7 +997,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -976,7 +1005,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -984,7 +1013,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -992,7 +1021,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>61</v>
       </c>
@@ -1002,20 +1031,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="48.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="2" width="48.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1023,7 +1052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -1031,7 +1060,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -1039,7 +1068,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>81</v>
       </c>
@@ -1047,7 +1076,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>83</v>
       </c>
@@ -1057,6 +1086,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>